<commit_message>
Excel Read Examples With DataProvider
</commit_message>
<xml_diff>
--- a/Students.xlsx
+++ b/Students.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\intellij-projects\core_java_santosh\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB66BEA-2634-468E-9DAD-2340A1BC80ED}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE423AF-DCC2-4441-8988-E941769B2D83}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{154082DA-BC81-40D5-AF76-6B7E267EB7C1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{154082DA-BC81-40D5-AF76-6B7E267EB7C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Students" sheetId="1" r:id="rId1"/>
-    <sheet name="Search" sheetId="3" r:id="rId2"/>
+    <sheet name="loginData" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>Name</t>
   </si>
@@ -64,16 +64,28 @@
     <t>830218321</t>
   </si>
   <si>
-    <t>Url</t>
-  </si>
-  <si>
-    <t>Automation</t>
-  </si>
-  <si>
-    <t>Mysql</t>
-  </si>
-  <si>
-    <t>Mobile Phones</t>
+    <t>userId</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>mngr629085</t>
+  </si>
+  <si>
+    <t>Ymaguty</t>
+  </si>
+  <si>
+    <t>312321sd</t>
+  </si>
+  <si>
+    <t>3213213sad</t>
+  </si>
+  <si>
+    <t>ewqesadas</t>
+  </si>
+  <si>
+    <t>wqewqewqe</t>
   </si>
 </sst>
 </file>
@@ -500,33 +512,55 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D49DE4-643D-4DB1-BD8A-F89C65327E27}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>